<commit_message>
Update the ICS score calculator workbook
Binary change made outside this session. Verified before committing
rather than pushed blind: _verify_ics_calculator.py reports 182 formulas
evaluated, 0 errors, 20/20 spot-checks against _draft_ics-scoring.md,
and 4/4 invariants holding (Standing >= Record across months 0-240,
Record(6)=25 so the gate opens exactly at Silver, Record at 12/36/60 =
50/75/100, Retention exactly 1.000 at the 30% allowance).

Still owed and unchanged by this commit: the gate is not modelled as a
mechanism. There is no pre-gate run counter, so scored rows still print
a pre-gate value (month 1 reads 4.2) where the design says no score
exists before the qualifying run and every displayed score is 25 or
higher. Rajesh's story also still opens at month 1 rather than at the
run. Listed in _draft_ics-scoring.md section 12.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/2-mechanism-design/Aurumix_ICS_Score_Calculator.xlsx
+++ b/deliverables/2-mechanism-design/Aurumix_ICS_Score_Calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://khiibaedu-my.sharepoint.com/personal/a_rehman_16863_khi_iba_edu_pk/Documents/Desktop/Aurumix/deliverables/2-mechanism-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_8413C6AA944726CF6264C4B54C5DCE3AF7434917" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F1D8809-AA7C-4FF1-817F-D54B2D729A40}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_8413C6AA944726CF6264C4B54C5DCE3AF7434917" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FD92643-3133-4958-8EEF-6BB240F77262}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="181">
   <si>
     <t>AURUMIX  ·  THE INVESTOR CONVICTION SCORE</t>
   </si>
@@ -215,9 +215,6 @@
     <t>Silver is permanent. Every tier above it is rented by conduct — which is the point.</t>
   </si>
   <si>
-    <t xml:space="preserve">  A WORKED STORY   —   Rajesh, USD 75 a month</t>
-  </si>
-  <si>
     <t>One missed payment and one real withdrawal, across five years. Follow the last two columns.</t>
   </si>
   <si>
@@ -573,6 +570,12 @@
   </si>
   <si>
     <t>The one number worth revisiting once we have real data is the withdrawal allowance. Everything else is structural.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  A WORKED STORY   —   Tony, USD 75 a month</t>
   </si>
 </sst>
 </file>
@@ -873,6 +876,989 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="95000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                    <a:prstClr val="black">
+                      <a:alpha val="40000"/>
+                    </a:prstClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Retention Score</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="51000"/>
+                    <a:satMod val="130000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="80000">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="93000"/>
+                    <a:satMod val="130000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="94000"/>
+                    <a:satMod val="135000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="16200000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="35000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+            <a:scene3d>
+              <a:camera prst="orthographicFront">
+                <a:rot lat="0" lon="0" rev="0"/>
+              </a:camera>
+              <a:lightRig rig="threePt" dir="t">
+                <a:rot lat="0" lon="0" rev="1200000"/>
+              </a:lightRig>
+            </a:scene3d>
+            <a:sp3d>
+              <a:bevelT w="63500" h="25400"/>
+            </a:sp3d>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>ICS!$B$37:$L$37</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>ICS!$B$38:$L$38</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.8571428571428571</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.71428571428571419</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.5714285714285714</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.4285714285714286</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.2857142857142857</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.14285714285714268</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-111F-4350-9D38-D2602ED7A8C4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="115"/>
+        <c:overlap val="-20"/>
+        <c:axId val="1467244095"/>
+        <c:axId val="736243279"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1467244095"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="736243279"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="736243279"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1467244095"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="222">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="34925" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>2324100</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D1F730E-08D9-628D-4C6F-1283C58D64F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1636,6 +2622,11 @@
         <v>32</v>
       </c>
     </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J40" t="s">
+        <v>179</v>
+      </c>
+    </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>33</v>
@@ -1801,7 +2792,7 @@
     </row>
     <row r="61" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
@@ -1819,36 +2810,36 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B64" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="21" t="s">
+      <c r="C64" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="C64" s="21" t="s">
+      <c r="D64" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D64" s="21" t="s">
+      <c r="E64" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="E64" s="21" t="s">
+      <c r="F64" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="F64" s="21" t="s">
+      <c r="G64" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="G64" s="21" t="s">
+      <c r="H64" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="H64" s="21" t="s">
+      <c r="I64" s="21" t="s">
         <v>69</v>
-      </c>
-      <c r="I64" s="21" t="s">
-        <v>70</v>
       </c>
       <c r="J64" s="21"/>
       <c r="K64" s="21" t="s">
@@ -1857,10 +2848,10 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B65" s="9" t="s">
         <v>71</v>
-      </c>
-      <c r="B65" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="C65" s="11">
         <v>1</v>
@@ -1898,10 +2889,10 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="B66" s="9" t="s">
         <v>73</v>
-      </c>
-      <c r="B66" s="9" t="s">
-        <v>74</v>
       </c>
       <c r="C66" s="11">
         <v>6</v>
@@ -1939,10 +2930,10 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="B67" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>76</v>
       </c>
       <c r="C67" s="11">
         <v>12</v>
@@ -1980,10 +2971,10 @@
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="C68" s="11">
         <v>24</v>
@@ -2021,10 +3012,10 @@
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="B69" s="9" t="s">
         <v>79</v>
-      </c>
-      <c r="B69" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="C69" s="11">
         <v>29</v>
@@ -2062,10 +3053,10 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="B70" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="B70" s="9" t="s">
-        <v>82</v>
       </c>
       <c r="C70" s="11">
         <v>35</v>
@@ -2103,10 +3094,10 @@
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B71" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>84</v>
       </c>
       <c r="C71" s="11">
         <v>36</v>
@@ -2144,10 +3135,10 @@
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B72" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="B72" s="9" t="s">
-        <v>86</v>
       </c>
       <c r="C72" s="11">
         <v>49</v>
@@ -2185,10 +3176,10 @@
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="B73" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="B73" s="9" t="s">
-        <v>88</v>
       </c>
       <c r="C73" s="11">
         <v>50</v>
@@ -2226,10 +3217,10 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="B74" s="9" t="s">
         <v>89</v>
-      </c>
-      <c r="B74" s="9" t="s">
-        <v>90</v>
       </c>
       <c r="C74" s="11">
         <v>59</v>
@@ -2267,10 +3258,10 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B75" s="9" t="s">
         <v>91</v>
-      </c>
-      <c r="B75" s="9" t="s">
-        <v>92</v>
       </c>
       <c r="C75" s="11">
         <v>60</v>
@@ -2308,27 +3299,27 @@
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="31" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="83" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B83" s="5"/>
       <c r="C83" s="5"/>
@@ -2346,96 +3337,96 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B86" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B86" s="21" t="s">
+      <c r="C86" s="21" t="s">
         <v>100</v>
-      </c>
-      <c r="C86" s="21" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B87" s="32">
         <v>42</v>
       </c>
       <c r="C87" s="24" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B88" s="32">
         <v>6</v>
       </c>
       <c r="C88" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B89" s="33">
         <v>30</v>
       </c>
       <c r="C89" s="24" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B90" s="33">
         <v>8</v>
       </c>
       <c r="C90" s="24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B91" s="33">
         <v>38</v>
       </c>
       <c r="C91" s="24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="B93" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B93" s="21" t="s">
+      <c r="C93" s="21" t="s">
         <v>113</v>
-      </c>
-      <c r="C93" s="21" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B94" s="34">
         <f>IF((B89+B90)&lt;=0,0,MAX(0,1-B91/(B89+B90)))</f>
         <v>0</v>
       </c>
       <c r="C94" s="24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
@@ -2447,7 +3438,7 @@
         <v>81.25</v>
       </c>
       <c r="C95" s="24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -2459,7 +3450,7 @@
         <v>50</v>
       </c>
       <c r="C96" s="24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
@@ -2471,72 +3462,72 @@
         <v>1</v>
       </c>
       <c r="C97" s="24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B98" s="35">
         <f>MIN(B95,B96)</f>
         <v>50</v>
       </c>
       <c r="C98" s="24" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B99" s="35">
         <f>IF(B87&gt;=$B$134,MAX($B$135,B98*B97),B98*B97)</f>
         <v>50</v>
       </c>
       <c r="C99" s="24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="100" spans="1:14" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A100" s="37" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B100" s="38" t="str">
         <f>VLOOKUP(B99,$A$52:$B$56,2,TRUE)</f>
         <v>Gold</v>
       </c>
       <c r="C100" s="24" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B101" s="39" t="str">
         <f>IF(B97&lt;1,"Selling",IF(B95&lt;B96,"Time — keep paying","Discipline — recent misses"))</f>
         <v>Discipline — recent misses</v>
       </c>
       <c r="C101" s="24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B102" s="40" t="str">
         <f>IF(B87&gt;=$B$134,"Yes — Silver secured","Not yet")</f>
         <v>Yes — Silver secured</v>
       </c>
       <c r="C102" s="24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="105" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B105" s="5"/>
       <c r="C105" s="5"/>
@@ -2554,44 +3545,44 @@
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B108" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C108" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="C108" s="21" t="s">
+      <c r="D108" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D108" s="21" t="s">
+      <c r="E108" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E108" s="21" t="s">
+      <c r="F108" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="F108" s="21" t="s">
+      <c r="G108" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="G108" s="21" t="s">
+      <c r="H108" s="21" t="s">
         <v>69</v>
-      </c>
-      <c r="H108" s="21" t="s">
-        <v>70</v>
       </c>
       <c r="I108" s="21" t="s">
         <v>40</v>
       </c>
       <c r="J108" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="41" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B109" s="42"/>
       <c r="C109" s="42"/>
@@ -2605,7 +3596,7 @@
     </row>
     <row r="110" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B110" s="11">
         <v>60</v>
@@ -2637,12 +3628,12 @@
         <v>Sovereign</v>
       </c>
       <c r="J110" s="24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B111" s="11">
         <v>60</v>
@@ -2674,12 +3665,12 @@
         <v>Sovereign</v>
       </c>
       <c r="J111" s="24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="112" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B112" s="11">
         <v>0</v>
@@ -2711,12 +3702,12 @@
         <v>No tier</v>
       </c>
       <c r="J112" s="24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="113" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A113" s="41" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B113" s="42"/>
       <c r="C113" s="42"/>
@@ -2730,7 +3721,7 @@
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A114" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B114" s="11">
         <v>36</v>
@@ -2762,12 +3753,12 @@
         <v>Platinum</v>
       </c>
       <c r="J114" s="24" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A115" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B115" s="11">
         <v>36</v>
@@ -2799,12 +3790,12 @@
         <v>Platinum</v>
       </c>
       <c r="J115" s="24" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A116" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B116" s="11">
         <v>36</v>
@@ -2836,12 +3827,12 @@
         <v>Gold</v>
       </c>
       <c r="J116" s="24" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A117" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B117" s="11">
         <v>36</v>
@@ -2873,12 +3864,12 @@
         <v>Silver</v>
       </c>
       <c r="J117" s="24" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B118" s="11">
         <v>60</v>
@@ -2910,12 +3901,12 @@
         <v>Silver</v>
       </c>
       <c r="J118" s="24" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="119" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A119" s="41" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B119" s="42"/>
       <c r="C119" s="42"/>
@@ -2929,7 +3920,7 @@
     </row>
     <row r="120" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B120" s="11">
         <v>120</v>
@@ -2961,12 +3952,12 @@
         <v>Platinum</v>
       </c>
       <c r="J120" s="24" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B121" s="11">
         <v>120</v>
@@ -2998,12 +3989,12 @@
         <v>Platinum</v>
       </c>
       <c r="J121" s="24" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A122" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B122" s="11">
         <v>120</v>
@@ -3035,12 +4026,12 @@
         <v>Gold</v>
       </c>
       <c r="J122" s="24" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B123" s="11">
         <v>120</v>
@@ -3072,12 +4063,12 @@
         <v>Silver</v>
       </c>
       <c r="J123" s="24" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="124" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A124" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B124" s="11">
         <v>120</v>
@@ -3109,12 +4100,12 @@
         <v>Silver</v>
       </c>
       <c r="J124" s="24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="125" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A125" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B125" s="11">
         <v>60</v>
@@ -3146,12 +4137,12 @@
         <v>Gold</v>
       </c>
       <c r="J125" s="24" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="128" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
@@ -3169,87 +4160,88 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="B129" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="C129" s="21" t="s">
         <v>165</v>
-      </c>
-      <c r="B129" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C129" s="21" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B130" s="32">
         <v>12</v>
       </c>
       <c r="C130" s="24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B131" s="32">
         <v>60</v>
       </c>
       <c r="C131" s="24" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B132" s="32">
         <v>12</v>
       </c>
       <c r="C132" s="24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B133" s="44">
         <v>0.3</v>
       </c>
       <c r="C133" s="24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B134" s="32">
         <v>6</v>
       </c>
       <c r="C134" s="24" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B135" s="32">
         <v>25</v>
       </c>
       <c r="C135" s="24" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>